<commit_message>
Wrap long item names within table cells
Added word-wrap:break-word to td and table-layout:fixed to enforce
column widths regardless of content length.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_inventory.xlsx
+++ b/sample_inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -678,6 +678,26 @@
         <v>175</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ART-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Extremt lång produktbenämning som verkligen inte får plats på en rad utan måste brytas och flöda ned på nästa rad i cellen</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PALL-C7</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add banner to first page, slim header on continuations
Page 1 of each pallet gets a full-width black banner with large
monospace location ID. Overflow pages get a slim rule with location,
page number and date. Also fixed scale accumulation bug where
painter.scale() was applied additively after each newPage().

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_inventory.xlsx
+++ b/sample_inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -698,6 +698,706 @@
         <v>42</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ART-101</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 1 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ART-102</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 2 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ART-103</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 3 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ART-104</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 4 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ART-105</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 5 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ART-106</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 6 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ART-107</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 7 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ART-108</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 8 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ART-109</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 9 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ART-110</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 10 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ART-111</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 11 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ART-112</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 12 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ART-113</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 13 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ART-114</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 14 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ART-115</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 15 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ART-116</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 16 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ART-117</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 17 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ART-118</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 18 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ART-119</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 19 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ART-120</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 20 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ART-121</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 21 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ART-122</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 22 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ART-123</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 23 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ART-124</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 24 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ART-125</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 25 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ART-126</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 26 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ART-127</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 27 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ART-128</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 28 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ART-129</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 29 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ART-130</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 30 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ART-131</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 31 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ART-132</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 32 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ART-133</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 33 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ART-134</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 34 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ART-135</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Testartikel nummer 35 med ganska lång benämning</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>PALL-D9</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>